<commit_message>
Update database configuration and enhance BffAuthController: Changed PostgreSQL credentials in docker-compose and appsettings.json, and added comments for clarity in BffAuthController methods to improve code readability.
</commit_message>
<xml_diff>
--- a/Explain Keycloak SSO.xlsx
+++ b/Explain Keycloak SSO.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dev\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Drive D\app\Factory Portal Root\app-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4C55610-7622-4758-B28C-E6E6514E010B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D6DC36-4324-418A-8061-4E72E6CAA46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{782F0D83-67FC-4482-B65E-F017EEE758C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{782F0D83-67FC-4482-B65E-F017EEE758C3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Code" sheetId="1" r:id="rId1"/>
+    <sheet name="Keycloak Setting" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,12 +39,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>มาที่ callback เพราะเป็น Redirect Uri</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1028,15 +1032,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>63499</xdr:colOff>
+      <xdr:colOff>63500</xdr:colOff>
       <xdr:row>227</xdr:row>
-      <xdr:rowOff>90713</xdr:rowOff>
+      <xdr:rowOff>101598</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>435429</xdr:colOff>
-      <xdr:row>245</xdr:row>
-      <xdr:rowOff>168692</xdr:rowOff>
+      <xdr:colOff>435430</xdr:colOff>
+      <xdr:row>246</xdr:row>
+      <xdr:rowOff>5406</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1059,8 +1063,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6749142" y="41274999"/>
-          <a:ext cx="10096501" cy="3343693"/>
+          <a:off x="7487557" y="39638512"/>
+          <a:ext cx="11170559" cy="3213065"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1077,15 +1081,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>54429</xdr:colOff>
+      <xdr:colOff>76201</xdr:colOff>
       <xdr:row>246</xdr:row>
-      <xdr:rowOff>163286</xdr:rowOff>
+      <xdr:rowOff>87086</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
-      <xdr:colOff>163286</xdr:colOff>
+      <xdr:colOff>185058</xdr:colOff>
       <xdr:row>255</xdr:row>
-      <xdr:rowOff>151783</xdr:rowOff>
+      <xdr:rowOff>75583</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1108,8 +1112,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6740072" y="44794715"/>
-          <a:ext cx="10441214" cy="1621354"/>
+          <a:off x="7500258" y="42933257"/>
+          <a:ext cx="11582400" cy="1556040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1126,39 +1130,485 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>63500</xdr:colOff>
+      <xdr:colOff>9072</xdr:colOff>
+      <xdr:row>257</xdr:row>
+      <xdr:rowOff>61687</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>441701</xdr:colOff>
+      <xdr:row>278</xdr:row>
+      <xdr:rowOff>152402</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Picture 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F590B1DC-E210-7F65-41D8-9C3659879A19}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="683986" y="44823744"/>
+          <a:ext cx="11231258" cy="3748315"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>13607</xdr:colOff>
       <xdr:row>258</xdr:row>
-      <xdr:rowOff>72571</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
+      <xdr:rowOff>68036</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>404655</xdr:colOff>
+      <xdr:row>310</xdr:row>
+      <xdr:rowOff>69607</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E5478A6-DD2B-7726-1133-590544301903}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12015107" y="45706393"/>
+          <a:ext cx="11059048" cy="9200000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>326572</xdr:colOff>
+      <xdr:row>214</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>529181</xdr:colOff>
+      <xdr:row>222</xdr:row>
+      <xdr:rowOff>170039</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4953429A-C773-D04A-7D47-08F510B105CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14328322" y="37855072"/>
+          <a:ext cx="4869859" cy="1585181"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>496129</xdr:colOff>
-      <xdr:row>279</xdr:row>
-      <xdr:rowOff>163286</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="28" name="Picture 27">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F590B1DC-E210-7F65-41D8-9C3659879A19}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="671286" y="46881142"/>
-          <a:ext cx="10157200" cy="3900715"/>
+      <xdr:colOff>618308</xdr:colOff>
+      <xdr:row>311</xdr:row>
+      <xdr:rowOff>71845</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>136071</xdr:colOff>
+      <xdr:row>334</xdr:row>
+      <xdr:rowOff>117631</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD650A24-841A-89B4-D2FB-D92EC3310C8B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11953058" y="55085524"/>
+          <a:ext cx="7518763" cy="4114321"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>297452</xdr:colOff>
+      <xdr:row>311</xdr:row>
+      <xdr:rowOff>108857</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>282364</xdr:colOff>
+      <xdr:row>325</xdr:row>
+      <xdr:rowOff>27214</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA2CF3DF-CB1F-567B-40FA-BBAE0D6DA79C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19633202" y="55122536"/>
+          <a:ext cx="3985412" cy="2394857"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38101</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>231679</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16F5CE47-25CB-54E8-CD9E-32944AEB9AF1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="708661" y="198120"/>
+          <a:ext cx="6228618" cy="2743200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>655320</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32571FBA-FC42-4B3F-7D7D-537CAC5328CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="655320" y="3177540"/>
+          <a:ext cx="6612255" cy="3657600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>107919</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0380BB7-6366-BE3C-451B-D26F13980772}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="670560" y="6972300"/>
+          <a:ext cx="6813519" cy="3657600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>30481</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>277942</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0B9A49E-EBB3-83A8-D2A6-C6E7337F3494}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="701041" y="10767060"/>
+          <a:ext cx="6953061" cy="3657600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>471280</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8CC9E605-55B1-A859-65A4-5F35E7EF570F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7909560" y="10812780"/>
+          <a:ext cx="7984600" cy="3657600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1492,9 +1942,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545EB084-C720-453D-AA26-8847E21194F3}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <dimension ref="S258"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData>
+    <row r="258" spans="19:19">
+      <c r="S258" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -1504,6 +1960,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50203A9-A8B1-4615-908D-509C3CE58E23}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{a280e33f-51f9-4eb7-bf6f-a0cb413b4c8b}" enabled="1" method="Standard" siteId="{d9cd485e-39bd-4cc9-9539-8c97631fbb71}" contentBits="1" removed="0"/>

</xml_diff>

<commit_message>
Update Explain Keycloak SSO.xlsx with new information and clarifications.
</commit_message>
<xml_diff>
--- a/Explain Keycloak SSO.xlsx
+++ b/Explain Keycloak SSO.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Drive D\app\Factory Portal Root\app-1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portal Web Demo\app-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D6DC36-4324-418A-8061-4E72E6CAA46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D5FE32-BBA8-4A72-BAA7-BFC5A935EAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{782F0D83-67FC-4482-B65E-F017EEE758C3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{782F0D83-67FC-4482-B65E-F017EEE758C3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Code" sheetId="1" r:id="rId1"/>
-    <sheet name="Keycloak Setting" sheetId="2" r:id="rId2"/>
+    <sheet name="Overview" sheetId="3" r:id="rId1"/>
+    <sheet name="Code" sheetId="1" r:id="rId2"/>
+    <sheet name="Keycloak Setting" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,6 +101,60 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>25401</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>53796</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA71AC85-2258-1B44-9C1D-ED2F59EC4A6C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="635001" y="184150"/>
+          <a:ext cx="3685995" cy="4019550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>101601</xdr:colOff>
       <xdr:row>2</xdr:row>
@@ -1375,7 +1430,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1941,11 +1996,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41549A5F-3FD7-43BA-AEC4-5C7BF3C1A742}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545EB084-C720-453D-AA26-8847E21194F3}">
   <dimension ref="S258"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="258" spans="19:19">
+    <row r="258" spans="19:19" x14ac:dyDescent="0.35">
       <c r="S258" t="s">
         <v>0</v>
       </c>
@@ -1960,10 +2025,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50203A9-A8B1-4615-908D-509C3CE58E23}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>